<commit_message>
conversion to markdown; reanalysis with timeline updates
</commit_message>
<xml_diff>
--- a/tables/Table S9.xlsx
+++ b/tables/Table S9.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael.studivan/Documents/GitHub/PortMiami-urban-coral-resilience/tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{95260E0A-3F5D-1B47-89E5-CBBC92154B04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7AAF8BB1-38CB-DC4F-B83C-5FBCD2BD1B65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6780" yWindow="3880" windowWidth="26440" windowHeight="15180" xr2:uid="{89A9F25D-FA09-224B-BFF8-AFA61B16EA13}"/>
+    <workbookView xWindow="6780" yWindow="3880" windowWidth="26440" windowHeight="15180" xr2:uid="{08BAF0B4-E839-4A48-A06D-28C50E9A8D77}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="88">
   <si>
     <t>Species</t>
   </si>
@@ -62,31 +62,136 @@
     <t>Orbicella faveolata</t>
   </si>
   <si>
-    <t>Bleaching vs OA</t>
+    <t>Urban vs Reef</t>
+  </si>
+  <si>
+    <t>DNA repair</t>
+  </si>
+  <si>
+    <t>Ofaveolata030677</t>
+  </si>
+  <si>
+    <t>Proximal promoter DNA-binding transcription activator activity, RNA polymerase II-specific</t>
+  </si>
+  <si>
+    <t>Urban</t>
   </si>
   <si>
     <t>Heat shock proteins</t>
   </si>
   <si>
+    <t>Ofaveolata032105</t>
+  </si>
+  <si>
+    <t>Heat shock 70 kDa protein 12A-like</t>
+  </si>
+  <si>
+    <t>Immune response</t>
+  </si>
+  <si>
+    <t>Ofaveolata006080</t>
+  </si>
+  <si>
+    <t>TNF receptor-associated factor BIRC3 binding domain</t>
+  </si>
+  <si>
+    <t>Oxidative stress/antioxidants</t>
+  </si>
+  <si>
+    <t>Ofaveolata003500</t>
+  </si>
+  <si>
+    <t>Amine oxidase</t>
+  </si>
+  <si>
+    <t>Ubiquitin-proteasome</t>
+  </si>
+  <si>
+    <t>Ofaveolata005888</t>
+  </si>
+  <si>
+    <t>Denticleless E3 ubiquitin protein ligase homolog (Drosophila)</t>
+  </si>
+  <si>
+    <t>Ofaveolata033710</t>
+  </si>
+  <si>
+    <t>Proteasomal ubiquitin-independent protein catabolic process</t>
+  </si>
+  <si>
+    <t>Ofaveolata033717</t>
+  </si>
+  <si>
+    <t>Proteasome activator complex subunit 4</t>
+  </si>
+  <si>
+    <t>Stress vs Control</t>
+  </si>
+  <si>
+    <t>Apoptosis/cell death</t>
+  </si>
+  <si>
+    <t>Ofaveolata029433</t>
+  </si>
+  <si>
+    <t>Caspase domain</t>
+  </si>
+  <si>
+    <t>OA, Bleaching, OA + Bleaching</t>
+  </si>
+  <si>
+    <t>Ofaveolata024079</t>
+  </si>
+  <si>
+    <t>RNA-directed 5'-3' RNA polymerase activity</t>
+  </si>
+  <si>
+    <t>Bleaching, OA + Bleaching</t>
+  </si>
+  <si>
+    <t>OA</t>
+  </si>
+  <si>
+    <t>Ofaveolata004474</t>
+  </si>
+  <si>
+    <t>Ubiquitin-like protein ligase activity</t>
+  </si>
+  <si>
+    <t>Ofaveolata007956</t>
+  </si>
+  <si>
+    <t>E3 ubiquitin-protein ligase synoviolin</t>
+  </si>
+  <si>
+    <t>Ofaveolata010796</t>
+  </si>
+  <si>
+    <t>Glutathione peroxidase activity</t>
+  </si>
+  <si>
+    <t>Ofaveolata013818</t>
+  </si>
+  <si>
+    <t>Glutathione S-transferase, N-terminal domain</t>
+  </si>
+  <si>
     <t>Ofaveolata021922</t>
   </si>
   <si>
-    <t>Suppression of tumorigenicity 13 (Hsp70 interacting protein)</t>
-  </si>
-  <si>
-    <t>Bleaching</t>
-  </si>
-  <si>
-    <t>OA</t>
-  </si>
-  <si>
-    <t>Ofaveolata023144</t>
-  </si>
-  <si>
-    <t>Ubiquitin homologues</t>
-  </si>
-  <si>
-    <t>Immune response</t>
+    <t>Suppression of tumorigenicity 13 (colon carcinoma) (Hsp70 interacting protein)</t>
+  </si>
+  <si>
+    <t>Ofaveolata024927</t>
+  </si>
+  <si>
+    <t>TNF receptor-associated factor</t>
+  </si>
+  <si>
+    <t>Ofaveolata032785</t>
+  </si>
+  <si>
+    <t>Glutathione S-transferase mu</t>
   </si>
   <si>
     <t>Ofaveolata000449</t>
@@ -95,15 +200,18 @@
     <t>Lactose-binding lectin l-2-like</t>
   </si>
   <si>
+    <t>Ofaveolata003751</t>
+  </si>
+  <si>
+    <t>Tachylectin</t>
+  </si>
+  <si>
     <t>Ofaveolata017142</t>
   </si>
   <si>
     <t>Galactose binding lectin domain</t>
   </si>
   <si>
-    <t>Oxidative stress/antioxidants</t>
-  </si>
-  <si>
     <t>Ofaveolata000053</t>
   </si>
   <si>
@@ -116,43 +224,82 @@
     <t>Peroxidase activity</t>
   </si>
   <si>
-    <t>Ofaveolata010796</t>
-  </si>
-  <si>
-    <t>Glutathione peroxidase activity</t>
-  </si>
-  <si>
     <t>Ofaveolata024342</t>
   </si>
   <si>
     <t>Animal haem peroxidase</t>
   </si>
   <si>
-    <t>OA + Bleaching vs OA</t>
-  </si>
-  <si>
-    <t>OA + Bleaching</t>
-  </si>
-  <si>
-    <t>Ofaveolata026158</t>
-  </si>
-  <si>
-    <t>Belongs to the glutathione peroxidase family</t>
+    <t>Ofaveolata016327</t>
+  </si>
+  <si>
+    <t>Ubiquitin-protein transferase activity</t>
+  </si>
+  <si>
+    <t>Ofaveolata026055</t>
+  </si>
+  <si>
+    <t>Ubiquitin-like protein-specific protease activity</t>
   </si>
   <si>
     <t>Siderastrea siderea</t>
   </si>
   <si>
-    <t>Ssiderea001633</t>
-  </si>
-  <si>
-    <t>Protein folding in endoplasmic reticulum</t>
-  </si>
-  <si>
-    <t>Ssiderea058218</t>
-  </si>
-  <si>
-    <t>Cytochrome C oxidase</t>
+    <t>Ssiderea60824</t>
+  </si>
+  <si>
+    <t>Reverse transcriptase (RNA-dependent DNA polymerase)</t>
+  </si>
+  <si>
+    <t>Ssiderea024906</t>
+  </si>
+  <si>
+    <t>Ssiderea026681</t>
+  </si>
+  <si>
+    <t>C-type lectin (CTL) or carbohydrate-recognition domain (CRD)</t>
+  </si>
+  <si>
+    <t>Ssiderea040857</t>
+  </si>
+  <si>
+    <t>Sialic acid binding Ig-like lectin 1, sialoadhesin</t>
+  </si>
+  <si>
+    <t>Ssiderea031312</t>
+  </si>
+  <si>
+    <t>Ssiderea000160</t>
+  </si>
+  <si>
+    <t>Mitochondrial membrane ATP synthase (F(1)F(0) ATP synthase or Complex V)</t>
+  </si>
+  <si>
+    <t>Ssiderea051176</t>
+  </si>
+  <si>
+    <t>Ubiquitin-2 like Rad60 SUMO-like</t>
+  </si>
+  <si>
+    <t>Ssiderea051703</t>
+  </si>
+  <si>
+    <t>Glutathione S-transferase, C-terminal domain</t>
+  </si>
+  <si>
+    <t>Ssiderea051704</t>
+  </si>
+  <si>
+    <t>Ssiderea012146</t>
+  </si>
+  <si>
+    <t>Ubiquitin-like modifier</t>
+  </si>
+  <si>
+    <t>Ssiderea028433</t>
+  </si>
+  <si>
+    <t>Histone H2A K63-linked ubiquitination</t>
   </si>
 </sst>
 </file>
@@ -233,7 +380,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -247,13 +394,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -588,14 +732,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50DF9426-58E3-0B44-BD50-AE0C0558AE0F}">
-  <dimension ref="A1:G19"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF2AE881-EC0C-CB4E-B8EB-5906ED8E139D}">
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="43.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="23.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -631,355 +777,627 @@
       <c r="C2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" ht="28" x14ac:dyDescent="0.2">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="4"/>
+      <c r="G3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="5" t="s">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="5" t="s">
+      <c r="F4" s="4"/>
+      <c r="G4" s="4" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="6"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="5" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="D5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="5" t="s">
+      <c r="E5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="6"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="5" t="s">
+      <c r="G5" s="4"/>
+    </row>
+    <row r="6" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="A6" s="5"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="D6" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="5" t="s">
+      <c r="E6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" s="5" t="s">
+    <row r="7" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="A7" s="5"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="5" t="s">
+      <c r="E7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>12</v>
       </c>
+      <c r="G7" s="4"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" s="5" t="s">
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="5" t="s">
+      <c r="E8" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>12</v>
       </c>
+      <c r="G8" s="4"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E9" s="5" t="s">
+      <c r="A9" s="5"/>
+      <c r="B9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F9" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="28" x14ac:dyDescent="0.2">
-      <c r="A10" s="6"/>
-      <c r="B10" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>30</v>
       </c>
+      <c r="D9" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
       <c r="C10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="G10" s="5" t="s">
+      <c r="D10" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="5"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="5"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F11" s="5" t="s">
+      <c r="D18" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G19" s="4"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" s="5"/>
+      <c r="B25" s="5"/>
+      <c r="C25" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" s="5"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="6"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="5" t="s">
+      <c r="D27" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" s="4"/>
+    </row>
+    <row r="28" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="A28" s="5"/>
+      <c r="B28" s="5"/>
+      <c r="C28" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D28" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G28" s="4"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" s="5"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" s="5"/>
+      <c r="B30" s="5"/>
+      <c r="C30" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F12" s="5" t="s">
+      <c r="D30" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="28" x14ac:dyDescent="0.2">
+      <c r="A31" s="5"/>
+      <c r="B31" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G31" s="4"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A32" s="5"/>
+      <c r="B32" s="5"/>
+      <c r="C32" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="6"/>
-      <c r="B13" s="6"/>
-      <c r="C13" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" s="5" t="s">
+      <c r="D32" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G32" s="4"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A33" s="5"/>
+      <c r="B33" s="5"/>
+      <c r="C33" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G33" s="4"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A34" s="5"/>
+      <c r="B34" s="5"/>
+      <c r="C34" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G34" s="4"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A35" s="5"/>
+      <c r="B35" s="5"/>
+      <c r="C35" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E13" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="6"/>
-      <c r="B14" s="6"/>
-      <c r="C14" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="6"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="6"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A17" s="6"/>
-      <c r="B17" s="6"/>
-      <c r="C17" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E17" s="5" t="s">
+      <c r="D35" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="F35" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F17" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="28" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="F19" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G19" s="8" t="s">
-        <v>31</v>
-      </c>
+      <c r="G35" s="4"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A36" s="6"/>
+      <c r="B36" s="6"/>
+      <c r="C36" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G36" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A2:A17"/>
-    <mergeCell ref="B2:B9"/>
-    <mergeCell ref="B10:B17"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="B18:B19"/>
+  <mergeCells count="6">
+    <mergeCell ref="A2:A25"/>
+    <mergeCell ref="B2:B8"/>
+    <mergeCell ref="B9:B25"/>
+    <mergeCell ref="A26:A36"/>
+    <mergeCell ref="B26:B30"/>
+    <mergeCell ref="B31:B36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>